<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-03 Le capitaine dans l'herbe
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-03.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-03.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut que son ours soit capitaine du seau-bateau, puis l'inviter au pique-nique. À chaque départ, elle reprend ce qu'il faut pour continuer.</t>
+          <t>Sur le radiateur, un bateau de papier sèche. Un pli de voile coupe la lumière. Victorina veut que l'ours soit capitaine du seau-bateau, maintenant. Au parc, elle saisit le seau trop lourd : il glisse. Elle refuse de foncer, reprend seau, manteau, capitaine. Au jardin, la gourde roule. Le pli de voile sur la nappe penche vers le dessous. À la maison, le pli touche une oreille.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur le radiateur, un bateau de papier sèche. Il sent encore la colle et la poussière. La voile est un peu froissée. C'est le bateau d'hier, Victorina. Il est tout chaud. Le radiateur l'a gardé. Une goutte glisse encore sur la vitre. Dehors, le ciel se déchire. La pluie s'en va. On met les chaussures ? Oui, papa. Avec l'ours. L'ours attend sur la chaise. Papa noue une chaussure. Ils ferment la porte. En ce moment, Victorina est au parc. Le soleil revient sur le bac à sable. Papa s'assoit sur le banc. Victorina a un seau jaune. Elle a un manteau bleu. L'ours est dans l'herbe. Le seau, c'est un bateau. Et l'ours ? Le capitaine. Je te vois. Victorina verse le sable. Ça fait chh. Le seau est lourd. Elle le pose près du bac. L'ours attend dans l'herbe mouillée. Le soleil baisse. On rentre. Le bateau reste ? Le bateau peut venir. C'est ton seau. On reprend ses affaires, avant de partir. Victorina prend le seau jaune. Il est lourd de sable. On le vide un peu. Le sable retombe. Chh. Il est plus léger. Le manteau est sur le banc. Elle le prend. Il est un peu froid. Et le capitaine ? Il est dans l'herbe. Victorina cherche. Une feuille couvre une oreille de l'ours. Il dormait. Elle le prend contre elle. Merci. On a tout. Ils rentrent. Plus tard, le jardin sent l'herbe coupée. Papa pose une nappe sur la table basse. C'est le pique-nique du capitaine. Il a faim. Victorina a une gourde. Elle a une casquette. L'ours est assis sur la nappe. J'ai soif. Bois un peu. L'eau fait glouglou. Une miette reste près de l'ours. On rentre. La soupe attend. Le capitaine aussi. Oui. Avant de partir, on reprend ses affaires. Victorina regarde la nappe. La gourde a roulé sous la table. La casquette est sur le banc du jardin. L'ours a encore la miette.</t>
+          <t>Sur la chaise, l'ours penche une oreille. Il regarde le radiateur, tiède. Un bateau de papier y dort. Il sent la colle, un peu la poussière. Un pli de voile coupe la lumière. La voile est froissée, toute petite. C'est le bateau d'hier, Victorina. Il est chaud, papa. Le radiateur l'a gardé. Dehors, le ciel se déchire. Une goutte glisse sur la vitre. La pluie s'en va. On met les chaussures ? Oui, papa. Avec l'ours, maintenant ! Papa noue une chaussure. L'ours attend contre son bras. Ils ferment la porte. Le parc sent la terre, mouillée. Le soleil revient sur le bac à sable. Papa s'assoit sur le banc. Victorina a un seau jaune. Elle a un manteau bleu. En ce moment, elle pose l'ours dans l'herbe. Le seau, c'est un bateau. Et l'ours ? Le capitaine. Je le mets là, tout de suite. Je te vois. Elle verse le sable dans le seau. Le seau devient lourd, très lourd. Elle le pose près du bac. L'ours attend dans l'herbe mouillée. Le soleil baisse. On rentre ? Le bateau reste ? Le bateau peut venir. Je le prends, maintenant ! Elle saisit le seau d'un coup. Le sable pèse trop. Le seau penche, puis glisse. Un filet de sable tombe sur ses chaussures. Oh. Le sourire quitte sa bouche. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux tirer, ou regarder ? Je veux le bateau. Victorina tire une dernière fois. Le seau reste trop lourd. Le manteau bleu reste sur le banc. L'ours reste dans l'herbe. Je reprends tout.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sur le radiateur, un bateau de papier sèche. Il sent encore la colle et la poussière. La voile est un peu froissée. C'est le bateau d'hier, Victorina. Il est tout chaud. Le radiateur l'a gardé. Une goutte glisse encore sur la vitre. Dehors, le ciel se déchire. La pluie s'en va. On met les chaussures ? Oui, papa. Avec l'ours. L'ours attend sur la chaise. Papa noue une chaussure. Ils ferment la porte. En ce moment, Victorina est au parc. Le soleil revient sur le bac à sable. Papa s'assoit sur le banc. Victorina a un seau jaune. Elle a un manteau bleu. L'ours est dans l'herbe. Le seau, c'est un bateau. Et l'ours ? Le capitaine. Je te vois. Victorina verse le sable. Ça fait chh. Le seau est lourd. Elle le pose près du bac. L'ours attend dans l'herbe mouillée. Le soleil baisse. On rentre. Le bateau reste ? Le bateau peut venir. C'est ton seau. On reprend ses affaires, avant de partir. Victorina prend le seau jaune. Il est lourd de sable. On le vide un peu. Le sable retombe. Chh. Il est plus léger. Le manteau est sur le banc. Elle le prend. Il est un peu froid. Et le capitaine ? Il est dans l'herbe. Victorina cherche. Une feuille couvre une oreille de l'ours. Il dormait. Elle le prend contre elle. Merci. On a tout. Ils rentrent. Plus tard, le jardin sent l'herbe coupée. Papa pose une nappe sur la table basse. C'est le pique-nique du capitaine. Il a faim. Victorina a une gourde. Elle a une casquette. L'ours est assis sur la nappe. J'ai soif. Bois un peu. L'eau fait glouglou. Une miette reste près de l'ours. On rentre. La soupe attend. Le capitaine aussi. Oui. Avant de partir, on reprend ses affaires. Victorina regarde la nappe. La gourde a roulé sous la table. La casquette est sur le banc du jardin. L'ours a encore la miette.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sur la chaise, l'ours penche une oreille. Il regarde le radiateur, tiède. Un bateau de papier y dort. Il sent la colle, un peu la poussière. Un &lt;emphasis level="moderate"&gt;pli de voile&lt;/emphasis&gt; coupe la lumière. La voile est froissée, toute petite. C'est le bateau d'hier, Victorina. Il est chaud, papa. Le radiateur l'a gardé. Dehors, le ciel se déchire. Une goutte glisse sur la vitre. La pluie s'en va. On met les chaussures ? Oui, papa. Avec l'ours, maintenant ! Papa noue une chaussure. L'ours attend contre son bras. Ils ferment la porte. Le parc sent la terre, mouillée. Le soleil revient sur le bac à sable. Papa s'assoit sur le banc. Victorina a un seau jaune. Elle a un manteau bleu. En ce moment, elle pose l'ours dans l'herbe. Le seau, c'est un bateau. Et l'ours ? Le capitaine. Je le mets là, tout de suite. Je te vois. Elle verse le sable dans le seau. Le seau devient lourd, très lourd. Elle le pose près du bac. L'ours attend dans l'herbe mouillée. Le soleil baisse. On rentre ? Le bateau reste ? Le bateau peut venir. Je le prends, maintenant ! Elle saisit le seau d'un coup. Le sable pèse trop. Le seau penche, puis glisse. Un filet de sable tombe sur ses chaussures. Oh. Le sourire quitte sa bouche. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux tirer, ou regarder ? Je veux le bateau. Victorina tire une dernière fois. Le seau reste trop lourd. Le manteau bleu reste sur le banc. L'ours reste dans l'herbe. Je reprends tout.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Zoé a joué longtemps au parc. Papa est sur le banc. Zoé a un seau jaune. Elle a un manteau bleu. Elle a son doudou ours. Le soleil baisse. Papa dit : on rentre. Papa dit : on va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires, avant de partir. Zoé s'arrête. Elle cherche le seau près du bac. Elle le prend. Elle cherche le manteau sur le banc. Elle le prend. Elle cherche le doudou dans l'herbe. L'herbe chatouille. Elle le prend. Maintenant Zoé a tout. Papa dit : merci. Plus tard, ils font un pique-nique au jardin. Zoé a une gourde. Elle a une casquette. Elle a encore le doudou. Papa dit : on rentre. Zoé se souvient. Avant de partir, on reprend ses affaires. Elle cherche la gourde. Elle la prend. Elle cherche la casquette. Elle la prend. Elle cherche le doudou. Elle le prend. Papa dit : tu as repris le geste. Même leçon, autre lieu. Zoé a tout. Ils marchent vers la maison. [pause]</t>
+          <t>Sur la chaise, l'ours penche une oreille. Il regarde le radiateur, tiède. Un bateau de papier y dort. Il sent la colle, un peu la poussière. Un &lt;emphasis&gt;pli de voile&lt;/emphasis&gt; coupe la lumière. La voile est froissée, toute petite. C'est le bateau d'hier, Victorina. Il est chaud, papa. Le radiateur l'a gardé. Dehors, le ciel se déchire. Une goutte glisse sur la vitre. La pluie s'en va. On met les chaussures ? Oui, papa. Avec l'ours, maintenant ! Papa noue une chaussure. L'ours attend contre son bras. Ils ferment la porte. Le parc sent la terre, mouillée. Le soleil revient sur le bac à sable. Papa s'assoit sur le banc. Victorina a un seau jaune. Elle a un manteau bleu. En ce moment, elle pose l'ours dans l'herbe. Le seau, c'est un bateau. Et l'ours ? Le capitaine. Je le mets là, tout de suite. Je te vois. Elle verse le sable dans le seau. Le seau devient lourd, très lourd. Elle le pose près du bac. L'ours attend dans l'herbe mouillée. Le soleil baisse. On rentre ? Le bateau reste ? Le bateau peut venir. Je le prends, maintenant ! Elle saisit le seau d'un coup. Le sable pèse trop. Le seau penche, puis glisse. Un filet de sable tombe sur ses chaussures. Oh. Le sourire quitte sa bouche. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux tirer, ou regarder ? Je veux le bateau. Victorina tire une dernière fois. Le seau reste trop lourd. Le manteau bleu reste sur le banc. L'ours reste dans l'herbe. Je reprends tout. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>pli de voile</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,88 +1326,71 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_capitaine_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Sur le radiateur, un bateau de papier sèche.
-narrateur|Il sent encore la colle et la poussière.
-narrateur|La voile est un peu froissée.
+          <t>narrateur|Sur la chaise, l'ours penche une oreille.
+narrateur|Il regarde le radiateur, tiède.
+narrateur|Un bateau de papier y dort.
+narrateur|Il sent la colle, un peu la poussière.
+narrateur|Un pli de voile coupe la lumière.
+narrateur|La voile est froissée, toute petite.
 papa|C'est le bateau d'hier, Victorina.
-enfant-f|Il est tout chaud.
+enfant-f|Il est chaud, papa.
 papa|Le radiateur l'a gardé.
-narrateur|Une goutte glisse encore sur la vitre.
 narrateur|Dehors, le ciel se déchire.
+narrateur|Une goutte glisse sur la vitre.
 papa|La pluie s'en va.
 papa|On met les chaussures ?
 enfant-f|Oui, papa.
-enfant-f|Avec l'ours.
-narrateur|L'ours attend sur la chaise.
+enfant-f|Avec l'ours, maintenant !
 narrateur|Papa noue une chaussure.
+narrateur|L'ours attend contre son bras.
 narrateur|Ils ferment la porte.
-narrateur|En ce moment, Victorina est au parc.
+narrateur|Le parc sent la terre, mouillée.
 narrateur|Le soleil revient sur le bac à sable.
 narrateur|Papa s'assoit sur le banc.
 narrateur|Victorina a un seau jaune.
 narrateur|Elle a un manteau bleu.
-narrateur|L'ours est dans l'herbe.
+narrateur|En ce moment, elle pose l'ours dans l'herbe.
 enfant-f|Le seau, c'est un bateau.
 papa|Et l'ours ?
 enfant-f|Le capitaine.
+enfant-f|Je le mets là, tout de suite.
 papa|Je te vois.
-narrateur|Victorina verse le sable.
-narrateur|Ça fait chh.
-narrateur|Le seau est lourd.
+narrateur|Elle verse le sable dans le seau.
+narrateur|Le seau devient lourd, très lourd.
 narrateur|Elle le pose près du bac.
 narrateur|L'ours attend dans l'herbe mouillée.
 papa|Le soleil baisse.
-papa|On rentre.
+papa|On rentre ?
 enfant-f|Le bateau reste ?
 papa|Le bateau peut venir.
-papa|C'est ton seau.
-papa|On reprend ses affaires, avant de partir.
-narrateur|Victorina prend le seau jaune.
-narrateur|Il est lourd de sable.
-papa|On le vide un peu.
-narrateur|Le sable retombe.
-narrateur|Chh.
-enfant-f|Il est plus léger.
-narrateur|Le manteau est sur le banc.
-narrateur|Elle le prend.
-narrateur|Il est un peu froid.
-enfant-f|Et le capitaine ?
-papa|Il est dans l'herbe.
-narrateur|Victorina cherche.
-narrateur|Une feuille couvre une oreille de l'ours.
-enfant-f|Il dormait.
-narrateur|Elle le prend contre elle.
-papa|Merci.
-papa|On a tout.
-narrateur|Ils rentrent.
-narrateur|Plus tard, le jardin sent l'herbe coupée.
-narrateur|Papa pose une nappe sur la table basse.
-papa|C'est le pique-nique du capitaine.
-enfant-f|Il a faim.
-narrateur|Victorina a une gourde.
-narrateur|Elle a une casquette.
-narrateur|L'ours est assis sur la nappe.
-enfant-f|J'ai soif.
-papa|Bois un peu.
-narrateur|L'eau fait glouglou.
-narrateur|Une miette reste près de l'ours.
-papa|On rentre.
-papa|La soupe attend.
-enfant-f|Le capitaine aussi.
-papa|Oui.
-papa|Avant de partir, on reprend ses affaires.
-narrateur|Victorina regarde la nappe.
-narrateur|La gourde a roulé sous la table.
-narrateur|La casquette est sur le banc du jardin.
-narrateur|L'ours a encore la miette.</t>
+enfant-f|Je le prends, maintenant !
+narrateur|Elle saisit le seau d'un coup.
+narrateur|Le sable pèse trop.
+narrateur|Le seau penche, puis glisse.
+narrateur|Un filet de sable tombe sur ses chaussures.
+enfant-f|Oh.
+narrateur|Le sourire quitte sa bouche.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux tirer, ou regarder ?
+enfant-f|Je veux le bateau.
+narrateur|Victorina tire une dernière fois.
+narrateur|Le seau reste trop lourd.
+narrateur|Le manteau bleu reste sur le banc.
+narrateur|L'ours reste dans l'herbe.
+enfant-f|Je reprends tout.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>radiateur,parc</t>
         </is>
       </c>
     </row>
@@ -1434,17 +1417,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Victorina ?</t>
+          <t>Le seau penche, trop lourd, près du bac. Avant de partir, que fait Victorina ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Victorina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le seau penche, trop lourd, près du bac. Avant de &lt;emphasis level="moderate"&gt;partir&lt;/emphasis&gt;, que fait Victorina ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir, que fait Zoé ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le seau penche, trop lourd, près du bac. Avant de &lt;emphasis&gt;partir&lt;/emphasis&gt;, que fait Victorina ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1507,18 +1490,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1533,38 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>partir</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1573,28 +1556,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=avant_de_partir_elle_reprend; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, que fait Victorina ?</t>
+          <t>narrateur|Le seau penche, trop lourd, près du bac.
+narrateur|Avant de partir, que fait Victorina ?</t>
         </is>
       </c>
     </row>
@@ -1621,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorina se penche. Elle prend la gourde sous la table. Elle s'était cachée. Oui. Comme le capitaine, tout à l'heure. Elle prend la casquette sur le banc. L'ours garde la miette dans sa patte. Je le prends. Elle le prend. Tu as repris tes affaires. Avant de partir. Les deux fois. Les deux fois. Bravo, Victorina. Papa plie la nappe. Ils marchent vers la maison. L'ours est contre elle. Tu tiens tout ? Oui, papa.</t>
+          <t>J'arrête de tirer. Elle pose le seau près du bac. Il est trop lourd. On le vide un peu ? Victorina penche le seau, sans presser. Le sable retombe en filet. Il est plus léger. Elle reprend le seau jaune. Le manteau bleu attend sur le banc. Elle le prend. Le tissu est un peu froid. Et le capitaine ? Il est dans l'herbe. Victorina cherche trop vite. L'herbe cache l'ours. Je ne le vois pas. Le sourire ne revient pas. Elle refuse de foncer. Elle s'arrête, les pieds dans l'herbe. Une feuille couvre une oreille. Il dormait. Elle prend l'ours contre elle. Merci, Victorina. Tu tiens tout ? Oui, papa. Le seau tape un peu sa jambe. Le manteau pèse sur son bras. L'ours sent l'herbe mouillée.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorina se penche. Elle prend la gourde sous la table. Elle s'était cachée. Oui. Comme le capitaine, tout à l'heure. Elle prend la casquette sur le banc. L'ours garde la miette dans sa patte. Je le prends. Elle le prend. Tu as repris tes affaires. Avant de partir. Les deux fois. Les deux fois. Bravo, Victorina. Papa plie la nappe. Ils marchent vers la maison. L'ours est contre elle. Tu tiens tout ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'arrête de tirer. Elle pose le seau près du bac. Il est trop lourd. On le vide un peu ? Victorina penche le seau, sans presser. Le sable retombe en filet. Il est plus léger. Elle reprend le seau jaune. Le manteau bleu attend sur le banc. Elle le prend. Le tissu est un peu froid. Et le &lt;emphasis level="moderate"&gt;capitaine&lt;/emphasis&gt; ? Il est dans l'herbe. Victorina cherche trop vite. L'herbe cache l'ours. Je ne le vois pas. Le sourire ne revient pas. Elle refuse de foncer. Elle s'arrête, les pieds dans l'herbe. Une feuille couvre une oreille. Il dormait. Elle prend l'ours contre elle. Merci, Victorina. Tu tiens tout ? Oui, papa. Le seau tape un peu sa jambe. Le manteau pèse sur son bras. L'ours sent l'herbe mouillée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Zoé a cherché. Elle a repris ses affaires. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir. Au parc, puis au pique-nique. [pause]</t>
+          <t>J'arrête de tirer. Elle pose le seau près du bac. Il est trop lourd. On le vide un peu ? Victorina penche le seau, sans presser. Le sable retombe en filet. Il est plus léger. Elle reprend le seau jaune. Le manteau bleu attend sur le banc. Elle le prend. Le tissu est un peu froid. Et le &lt;emphasis&gt;capitaine&lt;/emphasis&gt; ? Il est dans l'herbe. Victorina cherche trop vite. L'herbe cache l'ours. Je ne le vois pas. Le sourire ne revient pas. Elle refuse de foncer. Elle s'arrête, les pieds dans l'herbe. Une feuille couvre une oreille. Il dormait. Elle prend l'ours contre elle. Merci, Victorina. Tu tiens tout ? Oui, papa. Le seau tape un peu sa jambe. Le manteau pèse sur son bras. L'ours sent l'herbe mouillée. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1678,7 +1662,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1686,10 +1670,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1712,30 +1696,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>capitaine</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1744,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1760,35 +1744,44 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_reprend_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorina se penche.
-narrateur|Elle prend la gourde sous la table.
-enfant-f|Elle s'était cachée.
-papa|Oui.
-papa|Comme le capitaine, tout à l'heure.
-narrateur|Elle prend la casquette sur le banc.
-narrateur|L'ours garde la miette dans sa patte.
-enfant-f|Je le prends.
+          <t>enfant-f|J'arrête de tirer.
+narrateur|Elle pose le seau près du bac.
+enfant-f|Il est trop lourd.
+papa|On le vide un peu ?
+narrateur|Victorina penche le seau, sans presser.
+narrateur|Le sable retombe en filet.
+enfant-f|Il est plus léger.
+narrateur|Elle reprend le seau jaune.
+narrateur|Le manteau bleu attend sur le banc.
 narrateur|Elle le prend.
-papa|Tu as repris tes affaires.
-enfant-f|Avant de partir.
-enfant-f|Les deux fois.
-papa|Les deux fois.
-papa|Bravo, Victorina.
-narrateur|Papa plie la nappe.
-narrateur|Ils marchent vers la maison.
-narrateur|L'ours est contre elle.
+narrateur|Le tissu est un peu froid.
+enfant-f|Et le capitaine ?
+papa|Il est dans l'herbe.
+narrateur|Victorina cherche trop vite.
+narrateur|L'herbe cache l'ours.
+enfant-f|Je ne le vois pas.
+narrateur|Le sourire ne revient pas.
+narrateur|Elle refuse de foncer.
+narrateur|Elle s'arrête, les pieds dans l'herbe.
+narrateur|Une feuille couvre une oreille.
+enfant-f|Il dormait.
+narrateur|Elle prend l'ours contre elle.
+papa|Merci, Victorina.
 papa|Tu tiens tout ?
-enfant-f|Oui, papa.</t>
+enfant-f|Oui, papa.
+narrateur|Le seau tape un peu sa jambe.
+narrateur|Le manteau pèse sur son bras.
+narrateur|L'ours sent l'herbe mouillée.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>sable,manteau</t>
         </is>
       </c>
     </row>
@@ -1815,17 +1808,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils ouvrent la porte. Le bateau de papier est encore chaud. Il a attendu. Oui. Pose le seau à côté. Victorina pose le seau jaune. Les deux bateaux se touchent. Le petit et le grand. Tu poses la casquette sur la chaise ? Elle pose la casquette. Elle pose la gourde près de l'évier. L'ours garde la miette. Le capitaine a son goûter. Il peut naviguer demain. Demain, s'il fait beau. Victorina pose l'ours contre le bateau de papier. La voile froissée touche une oreille.</t>
+          <t>Plus tard, le jardin sent l'herbe coupée. Papa pose une nappe sur la table basse. C'est le pique-nique du capitaine. Il a faim, maintenant. Victorina a une gourde. Elle a une casquette. L'ours est assis sur la nappe. J'ai soif. Bois un peu. L'eau fait glouglou. Une miette reste près de l'ours. La soupe attend, à la maison. Le capitaine aussi. On y va, maintenant ! Elle saisit la gourde d'un coup. La gourde roule sous la table. Elle part ! Victorina veut se jeter dessous. La nappe glisse d'un coin. Le sourire disparaît. L'envie et l'inquiétude se bousculent. Pas comme le seau. Elle refuse de foncer. Personne ne dit la suite. Elle observe la nappe, puis la table. Un pli de voile y court, fin. Le même pli que sur le bateau. Le pli penche vers le dessous. Là. Tu suis ce pli ? Oui, papa. Elle se penche, sans presser. La gourde s'était cachée. Elle la prend. La casquette attend sur le banc du jardin. Elle la prend. L'ours garde la miette dans sa patte. Je le prends. Elle le prend contre elle.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils ouvrent la porte. Le bateau de papier est encore chaud. Il a attendu. Oui. Pose le seau à côté. Victorina pose le seau jaune. Les deux bateaux se touchent. Le petit et le grand. Tu poses la casquette sur la chaise ? Elle pose la casquette. Elle pose la gourde près de l'évier. L'ours garde la miette. Le capitaine a son goûter. Il peut naviguer demain. Demain, s'il fait beau. Victorina pose l'ours contre le bateau de papier. La voile froissée touche une oreille.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Plus tard, le jardin sent l'herbe coupée. Papa pose une nappe sur la table basse. C'est le pique-nique du capitaine. Il a faim, maintenant. Victorina a une gourde. Elle a une casquette. L'ours est assis sur la nappe. J'ai soif. Bois un peu. L'eau fait glouglou. Une miette reste près de l'ours. La soupe attend, à la maison. Le capitaine aussi. On y va, maintenant ! Elle saisit la gourde d'un coup. La gourde roule sous la table. Elle part ! Victorina veut se jeter dessous. La nappe glisse d'un coin. Le sourire disparaît. L'envie et l'inquiétude se bousculent. Pas comme le seau. Elle refuse de foncer. Personne ne dit la suite. Elle observe la nappe, puis la table. Un &lt;emphasis level="moderate"&gt;pli de voile&lt;/emphasis&gt; y court, fin. Le même pli que sur le bateau. Le pli penche vers le dessous. Là. Tu suis ce pli ? Oui, papa. Elle se penche, sans presser. La gourde s'était cachée. Elle la prend. La casquette attend sur le banc du jardin. Elle la prend. L'ours garde la miette dans sa patte. Je le prends. Elle le prend contre elle.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Zoé marche près de papa. Le doudou est dans son bras. [pause]</t>
+          <t>&lt;low-pitch&gt;Plus tard, le jardin sent l'herbe coupée. Papa pose une nappe sur la table basse. C'est le pique-nique du capitaine. Il a faim, maintenant. Victorina a une gourde. Elle a une casquette. L'ours est assis sur la nappe. J'ai soif. Bois un peu. L'eau fait glouglou. Une miette reste près de l'ours. La soupe attend, à la maison. Le capitaine aussi. On y va, maintenant ! Elle saisit la gourde d'un coup. La gourde roule sous la table. Elle part ! Victorina veut se jeter dessous. La nappe glisse d'un coin. Le sourire disparaît. L'envie et l'inquiétude se bousculent. Pas comme le seau. Elle refuse de foncer. Personne ne dit la suite. Elle observe la nappe, puis la table. Un &lt;emphasis&gt;pli de voile&lt;/emphasis&gt; y court, fin. Le même pli que sur le bateau. Le pli penche vers le dessous. Là. Tu suis ce pli ? Oui, papa. Elle se penche, sans presser. La gourde s'était cachée. Elle la prend. La casquette attend sur le banc du jardin. Elle la prend. L'ours garde la miette dans sa patte. Je le prends. Elle le prend contre elle.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1872,7 +1865,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1880,22 +1873,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1904,28 +1901,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>pli de voile</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1934,40 +1935,71 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_le_pli; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils ouvrent la porte.
-narrateur|Le bateau de papier est encore chaud.
-enfant-f|Il a attendu.
-papa|Oui.
-papa|Pose le seau à côté.
-narrateur|Victorina pose le seau jaune.
-narrateur|Les deux bateaux se touchent.
-enfant-f|Le petit et le grand.
-papa|Tu poses la casquette sur la chaise ?
-narrateur|Elle pose la casquette.
-narrateur|Elle pose la gourde près de l'évier.
-narrateur|L'ours garde la miette.
-papa|Le capitaine a son goûter.
-enfant-f|Il peut naviguer demain.
-papa|Demain, s'il fait beau.
-narrateur|Victorina pose l'ours contre le bateau de papier.
-narrateur|La voile froissée touche une oreille.</t>
+          <t>narrateur|Plus tard, le jardin sent l'herbe coupée.
+narrateur|Papa pose une nappe sur la table basse.
+papa|C'est le pique-nique du capitaine.
+enfant-f|Il a faim, maintenant.
+narrateur|Victorina a une gourde.
+narrateur|Elle a une casquette.
+narrateur|L'ours est assis sur la nappe.
+enfant-f|J'ai soif.
+papa|Bois un peu.
+narrateur|L'eau fait glouglou.
+narrateur|Une miette reste près de l'ours.
+papa|La soupe attend, à la maison.
+enfant-f|Le capitaine aussi.
+enfant-f|On y va, maintenant !
+narrateur|Elle saisit la gourde d'un coup.
+narrateur|La gourde roule sous la table.
+enfant-f|Elle part !
+narrateur|Victorina veut se jeter dessous.
+narrateur|La nappe glisse d'un coin.
+narrateur|Le sourire disparaît.
+narrateur|L'envie et l'inquiétude se bousculent.
+enfant-f|Pas comme le seau.
+narrateur|Elle refuse de foncer.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la nappe, puis la table.
+narrateur|Un pli de voile y court, fin.
+narrateur|Le même pli que sur le bateau.
+narrateur|Le pli penche vers le dessous.
+enfant-f|Là.
+papa|Tu suis ce pli ?
+enfant-f|Oui, papa.
+narrateur|Elle se penche, sans presser.
+narrateur|La gourde s'était cachée.
+narrateur|Elle la prend.
+narrateur|La casquette attend sur le banc du jardin.
+narrateur|Elle la prend.
+narrateur|L'ours garde la miette dans sa patte.
+enfant-f|Je le prends.
+narrateur|Elle le prend contre elle.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>jardin,nappe</t>
         </is>
       </c>
     </row>
@@ -1994,17 +2026,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai repris mes affaires. Avant de partir. Au parc, puis au jardin. Les deux bateaux restent côte à côte.</t>
+          <t>Ils ouvrent la porte. Le bateau de papier est tiède. Il a attendu. Pose le seau à côté ? Victorina pose le seau jaune. Les deux bateaux se touchent. Le petit et le grand. Elle pose la casquette sur la chaise. Elle pose la gourde près de l'évier. Victorina pose l'ours contre le bateau de papier. Le pli de voile touche une oreille. Le capitaine est rentré. Il a sa miette ? Oui. La voile froissée garde l'oreille au chaud.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai repris mes affaires. Avant de partir. Au parc, puis au jardin. Les deux bateaux restent côte à côte.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils ouvrent la porte. Le bateau de papier est tiède. Il a attendu. Pose le seau à côté ? Victorina pose le seau jaune. Les deux bateaux se touchent. Le petit et le grand. Elle pose la casquette sur la chaise. Elle pose la gourde près de l'évier. Victorina pose l'ours contre le bateau de papier. Le &lt;emphasis level="moderate"&gt;pli de voile&lt;/emphasis&gt; touche une oreille. Le capitaine est rentré. Il a sa miette ? Oui. La voile froissée garde l'oreille au chaud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils ouvrent la porte. Le bateau de papier est tiède. Il a attendu. Pose le seau à côté ? Victorina pose le seau jaune. Les deux bateaux se touchent. Le petit et le grand. Elle pose la casquette sur la chaise. Elle pose la gourde près de l'évier. Victorina pose l'ours contre le bateau de papier. Le &lt;emphasis&gt;pli de voile&lt;/emphasis&gt; touche une oreille. Le capitaine est rentré. Il a sa miette ? Oui. La voile froissée garde l'oreille au chaud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2051,18 +2083,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2071,12 +2103,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2085,17 +2117,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>pli de voile</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2104,11 +2140,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2117,27 +2153,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=le_pli_de_voile_touche_une_oreille; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai repris mes affaires.
-papa|Avant de partir.
-papa|Au parc, puis au jardin.
-narrateur|Les deux bateaux restent côte à côte.</t>
+          <t>narrateur|Ils ouvrent la porte.
+narrateur|Le bateau de papier est tiède.
+enfant-f|Il a attendu.
+papa|Pose le seau à côté ?
+narrateur|Victorina pose le seau jaune.
+narrateur|Les deux bateaux se touchent.
+enfant-f|Le petit et le grand.
+narrateur|Elle pose la casquette sur la chaise.
+narrateur|Elle pose la gourde près de l'évier.
+narrateur|Victorina pose l'ours contre le bateau de papier.
+narrateur|Le pli de voile touche une oreille.
+enfant-f|Le capitaine est rentré.
+papa|Il a sa miette ?
+enfant-f|Oui.
+narrateur|La voile froissée garde l'oreille au chaud.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>porte,bateau</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2250,6 +2306,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>